<commit_message>
Remove catalog image badge and sync catalog photos
</commit_message>
<xml_diff>
--- a/sutra-catalog-update.xlsx
+++ b/sutra-catalog-update.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rbf4915b453e74247"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" r:id="Rcecd209f8a43456b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,7 +286,7 @@
     <x:col min="4" max="4" width="13.130000114440918" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="27.5" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="55" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="37.5" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="22.5" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18.75" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="18.75" hidden="0" customWidth="1"/>
@@ -351,7 +351,9 @@
       <x:c r="F2" s="7" t="str">
         <x:v>Light as air and easy to wear, this mulmul cotton saree brings quiet elegance to everyday dressing. A comfortable choice for work, relaxed outings, and the simple moments in between.</x:v>
       </x:c>
-      <x:c r="G2" s="7" t="str"/>
+      <x:c r="G2" s="7" t="str">
+        <x:v>https://drive.google.com/uc?export=view&amp;id=1vOXNV6BurNDLOBR3GDOxMbf2pEoQ-gWm</x:v>
+      </x:c>
       <x:c r="H2" s="7" t="str">
         <x:v>Soft Mulmul Cotton</x:v>
       </x:c>
@@ -381,7 +383,9 @@
       <x:c r="F3" s="7" t="str">
         <x:v>Made for long, easy days, this airy mulmul cotton saree keeps comfort at the heart of the drape. Its understated look moves naturally from office hours to casual outings.</x:v>
       </x:c>
-      <x:c r="G3" s="7" t="str"/>
+      <x:c r="G3" s="7" t="str">
+        <x:v>https://drive.google.com/uc?export=view&amp;id=1RUYGmGhsnOnMae4Jk-2c52-dg6nNIaaE</x:v>
+      </x:c>
       <x:c r="H3" s="7" t="str">
         <x:v>Soft Mulmul Cotton</x:v>
       </x:c>
@@ -411,7 +415,9 @@
       <x:c r="F4" s="7" t="str">
         <x:v>A delicate lotus motif adds a thoughtful detail to this airy mulmul cotton saree. Lightweight and breathable, it is made for everyday wear, office days, and relaxed occasions. Saree only, blouse piece not included.</x:v>
       </x:c>
-      <x:c r="G4" s="7" t="str"/>
+      <x:c r="G4" s="7" t="str">
+        <x:v>https://drive.google.com/uc?export=view&amp;id=1IuqVeNGpMc3oGEh8Rup9dbH6oVpQi8Tv</x:v>
+      </x:c>
       <x:c r="H4" s="7" t="str">
         <x:v>Soft Mulmul Cotton</x:v>
       </x:c>
@@ -441,7 +447,9 @@
       <x:c r="F5" s="7" t="str">
         <x:v>An airy mulmul cotton drape with a clean, timeless feel. Soft, breathable, and easy to style, it is a comfortable companion for everyday wear and casual occasions.</x:v>
       </x:c>
-      <x:c r="G5" s="7" t="str"/>
+      <x:c r="G5" s="7" t="str">
+        <x:v>https://drive.google.com/uc?export=view&amp;id=1rVw4WbuA21J5a104iiMJEE7hLbcSvExK</x:v>
+      </x:c>
       <x:c r="H5" s="7" t="str">
         <x:v>Soft Mulmul Cotton</x:v>
       </x:c>
@@ -471,7 +479,9 @@
       <x:c r="F6" s="7" t="str">
         <x:v>Fine rose threadwork brings a soft accent to this lightweight mulmul cotton saree. Breathable and comfortable through the day, it suits office wear, casual outings, and everyday dressing. Saree only, blouse piece not included.</x:v>
       </x:c>
-      <x:c r="G6" s="7" t="str"/>
+      <x:c r="G6" s="7" t="str">
+        <x:v>https://drive.google.com/uc?export=view&amp;id=16ruUWdM7FHGKN7plfo-iq3RuBCMrJ1hi</x:v>
+      </x:c>
       <x:c r="H6" s="7" t="str">
         <x:v>Soft Mulmul Cotton</x:v>
       </x:c>
@@ -501,7 +511,9 @@
       <x:c r="F7" s="7" t="str">
         <x:v>A simple cotton drape with a timeless feel. Soft and comfortable to wear, this plain saree brings understated elegance to everyday dressing.</x:v>
       </x:c>
-      <x:c r="G7" s="7" t="str"/>
+      <x:c r="G7" s="7" t="str">
+        <x:v>https://drive.google.com/uc?export=view&amp;id=1vYBi1bbSzGYHAqMnsTEzOShPmd-Vas7G</x:v>
+      </x:c>
       <x:c r="H7" s="7" t="str">
         <x:v>Cotton</x:v>
       </x:c>
@@ -531,7 +543,9 @@
       <x:c r="F8" s="7" t="str">
         <x:v>Soft cotton meets the traditional leena bhutta motif in a saree made for comfortable everyday wear. Its subtle detailing adds a little heritage to an easy, graceful drape.</x:v>
       </x:c>
-      <x:c r="G8" s="7" t="str"/>
+      <x:c r="G8" s="7" t="str">
+        <x:v>https://drive.google.com/uc?export=view&amp;id=1GwjE1A3zYFL6c7W5thwZFqplNT-HMXiE</x:v>
+      </x:c>
       <x:c r="H8" s="7" t="str">
         <x:v>Cotton</x:v>
       </x:c>
@@ -561,7 +575,9 @@
       <x:c r="F9" s="7" t="str">
         <x:v>Finished with lotus embroidery, this mulmul cotton saree pairs a classic detail with a light, comfortable drape. An easy choice for daily wear, office days, and casual occasions.</x:v>
       </x:c>
-      <x:c r="G9" s="7" t="str"/>
+      <x:c r="G9" s="7" t="str">
+        <x:v>https://drive.google.com/uc?export=view&amp;id=1IuqVeNGpMc3oGEh8Rup9dbH6oVpQi8Tv</x:v>
+      </x:c>
       <x:c r="H9" s="7" t="str">
         <x:v>Soft Mulmul Cotton</x:v>
       </x:c>
@@ -591,7 +607,9 @@
       <x:c r="F10" s="7" t="str">
         <x:v>Delicate rose threadwork gives this breathable mulmul cotton saree a graceful finish. Light and comfortable through the day, it is an easy choice for office wear, everyday dressing, and casual outings. Saree only, blouse piece not included.</x:v>
       </x:c>
-      <x:c r="G10" s="7" t="str"/>
+      <x:c r="G10" s="7" t="str">
+        <x:v>https://drive.google.com/uc?export=view&amp;id=1gj9TFU2QgXSFd_zN37RwLhwgQFADtQak</x:v>
+      </x:c>
       <x:c r="H10" s="7" t="str">
         <x:v>Soft Mulmul Cotton</x:v>
       </x:c>

</xml_diff>